<commit_message>
intel: Sept 11 biopharma brief; resolve two early approvals, add 8 catalysts
Brief: camizestrant ctDNA-triggered accelerated approval (a Sep 4 miss),
Isembyld/apitegromab SMA approval 19 days early, Joenja pediatric APDS
approval 43 days early after a CRL.

Watchlist 46 -> 54 rows:
- apitegromab and leniolisib resolved to approved with actual_date 2026-09-11
- Telix TLX101-Px left upcoming; PDUFA passed with no announcement
- Winrevair corrected from sNDA to sBLA (BLA 761363)
- new: camizestrant, sevabertinib, atogepant LUNA, zipalertinib, inaxaplin,
  VRBPAC Oct 1, MR-141, INO-3107
- first two womens_health_relevant=true rows (camizestrant, atogepant)
- deduped pdufa.bio's split MR-141/phentolamine listing; corrected INO-3107
  indication from CIN to RRP

intel:sweep:check passes: 54 rows, no duplicates, no schema violations, sorted.
</commit_message>
<xml_diff>
--- a/intel/biopharma-weekly/catalysts.xlsx
+++ b/intel/biopharma-weekly/catalysts.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalysts" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Catalysts'!$A$1:$K$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,11 +33,40 @@
       <sz val="11"/>
     </font>
     <font>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <color rgb="000563C1"/>
+      <sz val="10"/>
       <u val="single"/>
     </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007F6000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00833C0C"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +90,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
@@ -70,7 +104,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -78,48 +112,37 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D9D9D9"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9D9D9"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -487,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -503,7 +526,7 @@
     <col width="55" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>date_added</t>
@@ -586,32 +609,32 @@
           <t>NUVL</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>zidesamtinib</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>ROS1 TKI</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>ROS1+ NSCLC</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
         <is>
           <t>Approved Jul 22 2026 as Jideytro; prior Sep 18 PDUFA row was stale</t>
         </is>
@@ -643,17 +666,17 @@
           <t>—</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>biosimilar container closure systems draft guidance</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>biosimilars</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -663,12 +686,12 @@
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>Draft guidance on device presentations for biosimilars; comments due Oct 2 2026</t>
         </is>
@@ -700,17 +723,17 @@
           <t>AMGN</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Tavneos (avacopan)</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>complement C5aR antagonist</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>ANCA-associated vasculitis</t>
         </is>
@@ -720,12 +743,12 @@
           <t>withdrawn</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>EU authorization revoked Aug 4 over trial-data integrity; FDA withdrawal hearing pending</t>
         </is>
@@ -757,32 +780,32 @@
           <t>private</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>177Lu-edotreotide</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>radioligand therapy</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>gastroenteropancreatic neuroendocrine tumors</t>
         </is>
       </c>
-      <c r="I5" s="7" t="inlineStr">
+      <c r="I5" s="8" t="inlineStr">
         <is>
           <t>CRL</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
         <is>
           <t>CRL issued Aug 7</t>
         </is>
@@ -814,32 +837,32 @@
           <t>BMY</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>Zenbexus (iberdomide)</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>CELMoD</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>relapsed/refractory multiple myeloma</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
         <is>
           <t>First CELMoD; accelerated approval 4 days before Aug 17 PDUFA</t>
         </is>
@@ -871,32 +894,32 @@
           <t>LNTH</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>Tauklarify (florquinitau F 18)</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>tau PET imaging agent</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>Alzheimer's disease evaluation</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
         <is>
           <t>Novel tau PET tracer</t>
         </is>
@@ -928,32 +951,32 @@
           <t>EYPT</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="3" t="inlineStr">
         <is>
           <t>DURAVYU (vorolanib insert)</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>intravitreal TKI insert</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>wet AMD</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="I8" s="8" t="inlineStr">
         <is>
           <t>negative</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
         <is>
           <t>LUGANO missed primary endpoint in full dataset; shares -58%</t>
         </is>
@@ -985,32 +1008,32 @@
           <t>ARGX</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>Vyvgart Hytrulo (efgartigimod)</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>FcRn antagonist</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>autoimmune myositis</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
         <is>
           <t>ALKIVIA Ph3 met primary (p=0.0011); first Ph3 win in IMNM subtype</t>
         </is>
@@ -1042,32 +1065,32 @@
           <t>AMLX</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="3" t="inlineStr">
         <is>
           <t>avexitide</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>GLP-1 receptor antagonist</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>post-bariatric hypoglycemia</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
         <is>
           <t>LUCIDITY Ph3: 55% reduction in hypoglycemic events; shares +63%</t>
         </is>
@@ -1099,32 +1122,32 @@
           <t>MRNA</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>intismeran autogene + Keytruda</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>individualized mRNA neoantigen therapy</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>resected high-risk melanoma</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
         <is>
           <t>INTerpath-001 met RFS + DMFS at interim; first positive Ph3 for individualized mRNA cancer therapy</t>
         </is>
@@ -1156,32 +1179,32 @@
           <t>REGN</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>Pasatru (garetosmab)</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>activin-A antibody</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>fibrodysplasia ossificans progressiva</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
         <is>
           <t>Approved ~2 weeks ahead of Aug 31 PDUFA; second-ever FOP therapy</t>
         </is>
@@ -1213,32 +1236,32 @@
           <t>RARE</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" s="3" t="inlineStr">
         <is>
           <t>GENGLYCOS (pariglasgene brecaparvovec)</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>AAV gene therapy</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>glycogen storage disease type Ia</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
         <is>
           <t>First therapy for GSDIa; accelerated approval 4 days before Aug 23 PDUFA</t>
         </is>
@@ -1270,32 +1293,32 @@
           <t>BIIB</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" s="3" t="inlineStr">
         <is>
           <t>lecanemab SC starting dose</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>anti-amyloid antibody</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Alzheimer's disease</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
         <is>
           <t>Approved Jul 13 2026 as Leqembi IQLIK (first at-home starting dose); US launch late Aug 2026</t>
         </is>
@@ -1327,32 +1350,32 @@
           <t>JAZZ</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>Ziihera (zanidatamab)</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>HER2 bispecific antibody</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>1L HER2+ gastroesophageal adenocarcinoma</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
         <is>
           <t>Approved Aug 25 2026 for 1L HER2+ GEA with and without tislelizumab; median OS 26.4 months</t>
         </is>
@@ -1384,32 +1407,32 @@
           <t>JNJ</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>Imaavy (nipocalimab)</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>FcRn blocker</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>warm autoimmune hemolytic anemia (12+)</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
         <is>
           <t>First drug approved for wAIHA</t>
         </is>
@@ -1441,32 +1464,32 @@
           <t>RVMD</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="F17" s="3" t="inlineStr">
         <is>
           <t>Rasonque (daraxonrasib)</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>RAS(ON) multi-selective inhibitor</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>metastatic pancreatic adenocarcinoma (2L+)</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
         <is>
           <t>First targeted therapy for metastatic pancreatic cancer; roughly doubled survival in pivotal trial</t>
         </is>
@@ -1498,32 +1521,32 @@
           <t>GILD</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" s="3" t="inlineStr">
         <is>
           <t>bictegravir/lenacapavir</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>HIV single-tablet regimen</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>HIV-1</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
         <is>
           <t>Approved Aug 27 2026 as Bixlenvo; smallest once-daily single-tablet HIV regimen</t>
         </is>
@@ -1555,32 +1578,32 @@
           <t>CYTK</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="3" t="inlineStr">
         <is>
           <t>aficamten (ACACIA-HCM)</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>cardiac myosin inhibitor</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>non-obstructive hypertrophic cardiomyopathy</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
         <is>
           <t>Full Ph3 results at ESC + NEJM; met dual primaries (KCCQ-CSS p=0.021; pVO2 p=0.003); sNDA planned Q4 2026</t>
         </is>
@@ -1612,32 +1635,32 @@
           <t>LLY</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" s="3" t="inlineStr">
         <is>
           <t>Mounjaro (tirzepatide) CV label</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>GIP/GLP-1 receptor agonist</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>MACE risk reduction in type 2 diabetes</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
         <is>
           <t>Label expansion on SURPASS-CVOT (&gt;13000 patients ~4-year follow-up)</t>
         </is>
@@ -1669,32 +1692,32 @@
           <t>NVS</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>rapcabtagene autoleucel (rap-cel)</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>autologous CD19 CAR-T</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>rheumatic and neurological autoimmune disease</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I21" s="8" t="inlineStr">
         <is>
           <t>negative</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
         <is>
           <t>8 trials paused after 3 patient deaths from severe immune reaction; oncology trials unaffected; BMS halted a comparable autoimmune CAR-T program the same week</t>
         </is>
@@ -1726,32 +1749,32 @@
           <t>NVS</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>remibrutinib</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>BTK inhibitor</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>relapsing multiple sclerosis</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K22" s="5" t="inlineStr">
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
         <is>
           <t>REMODEL-1/-2 met primary ARR vs teriflunomide plus all key secondaries; no BTK liver signal; filing planned, full data ~October</t>
         </is>
@@ -1783,32 +1806,32 @@
           <t>6446.TW</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Besremi (ropeginterferon alfa-2b) sBLA</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>interferon</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>essential thrombocythemia</t>
         </is>
       </c>
-      <c r="I23" s="3" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>approved</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K23" s="5" t="inlineStr">
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>Approved Aug 31 2026; first new ET agent in the US since anagrelide (1997); SURPASS-ET Ph3</t>
         </is>
@@ -1827,47 +1850,47 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>approval</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>American Regent (Daiichi Sankyo)</t>
+          <t>Alumis</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Injectafer (ferric carboxymaltose) boxed warning</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>IV iron replacement</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>iron deficiency anemia</t>
-        </is>
-      </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>Labeling revision adds boxed warning for severe prolonged symptomatic hypophosphatemia; follows Aug 13 citizen-petition grant; relevant to OB/GYN IV iron use</t>
+          <t>ALMS</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>envudeucitinib</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>TYK2 inhibitor</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>systemic lupus erythematosus</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>negative</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>Ph2b LUMUS missed primary and key secondary; high-interferon subgroup active; Ph3 still planned</t>
         </is>
       </c>
     </row>
@@ -1884,47 +1907,47 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>readout</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Alumis</t>
+          <t>American Regent (Daiichi Sankyo)</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>ALMS</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>envudeucitinib</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>TYK2 inhibitor</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>systemic lupus erythematosus</t>
-        </is>
-      </c>
-      <c r="I25" s="7" t="inlineStr">
-        <is>
-          <t>negative</t>
-        </is>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>Ph2b LUMUS missed primary and key secondary; high-interferon subgroup active; Ph3 still planned</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Injectafer (ferric carboxymaltose) boxed warning</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>IV iron replacement</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>iron deficiency anemia</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Labeling revision adds boxed warning for severe prolonged symptomatic hypophosphatemia; follows Aug 13 citizen-petition grant; relevant to OB/GYN IV iron use</t>
         </is>
       </c>
     </row>
@@ -1954,32 +1977,32 @@
           <t>SMMT</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="F26" s="3" t="inlineStr">
         <is>
           <t>ivonescimab</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>PD-1/VEGF bispecific antibody</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>PD-L1-positive advanced NSCLC</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K26" s="5" t="inlineStr">
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
         <is>
           <t>HARMONi-2 (China) showed statistically significant OS benefit vs pembrolizumab monotherapy; first PD-1/VEGF bispecific to beat Keytruda on OS</t>
         </is>
@@ -2011,32 +2034,32 @@
           <t>RARE</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>apazunersen (GTX-102)</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>antisense oligonucleotide</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H27" s="3" t="inlineStr">
         <is>
           <t>Angelman syndrome</t>
         </is>
       </c>
-      <c r="I27" s="7" t="inlineStr">
+      <c r="I27" s="8" t="inlineStr">
         <is>
           <t>negative</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="inlineStr">
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
         <is>
           <t>Ph3 Aspire missed primary (Bayley-4 cognitive) and key secondary (MRI net response); no treated-vs-control differences; company weighing significant cost cuts ahead of Sep 19 UX111 PDUFA</t>
         </is>
@@ -2068,32 +2091,32 @@
           <t>ABBV</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" s="3" t="inlineStr">
         <is>
           <t>etentamig (ABBV-383)</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>BCMA/CD3 bispecific antibody</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>relapsed/refractory multiple myeloma</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>positive</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K28" s="5" t="inlineStr">
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
         <is>
           <t>Positive Ph3 CERVINO reported the same day AbbVie closed its $10.9B Apogee acquisition at $135.11/share</t>
         </is>
@@ -2102,171 +2125,171 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Telix</t>
+          <t>AstraZeneca</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>TLX</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>TLX101-Px</t>
-        </is>
-      </c>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>PET imaging agent</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>glioma imaging</t>
-        </is>
-      </c>
-      <c r="I29" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K29" s="5" t="inlineStr">
-        <is>
-          <t>Radiopharma imaging momentum</t>
+          <t>AZN</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Etcamah (camizestrant)</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>oral SERD</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>ESR1-mutated HR+/HER2- advanced or metastatic breast cancer</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Accelerated approval Sep 4 2026, 75 mg once daily with abemaciclib, palbociclib or ribociclib. First US approval of a cancer therapy triggered by a resistance mutation detected in blood before imaging shows progression - moves the regulatory unit of analysis from radiographic progression to a ctDNA signal, with read-through to liquid-biopsy assays as companion-diagnostic gatekeepers. Narrower than a general ctDNA endpoint precedent: accelerated approval in an on-treatment resistance population, confirmatory obligation still governs. No published NICE appraisal and no establishable MHRA date as of Sep 8 2026. MISSED by the Sep 4 brief, which published at 5:04 PM ET the same day</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>CHMP</t>
+          <t>approval</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>EMA</t>
+          <t>Bayer</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>CHMP monthly meeting</t>
-        </is>
-      </c>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I30" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K30" s="5" t="inlineStr">
-        <is>
-          <t>Sept 14-17; new opinions resume after August written procedure</t>
+          <t>BAYRY</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Hyrnuo (sevabertinib)</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>HER2-selective tyrosine kinase inhibitor</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>first-line HER2-mutant locally advanced or metastatic non-squamous NSCLC</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Accelerated approval Sep 9 2026 following priority review; first-line option in HER2-mutant NSCLC. Third FDA approval inside the Sep 5-11 week</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>AdComm</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>FDA</t>
+          <t>AbbVie</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Pediatric Advisory Committee</t>
-        </is>
-      </c>
-      <c r="G31" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K31" s="5" t="inlineStr">
-        <is>
-          <t>Virtual session</t>
+          <t>ABBV</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>atogepant (QULIPTA/AQUIPTA)</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>oral CGRP receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>preventive treatment of menstrual migraine</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>positive</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3 LUNA topline met the primary endpoint and all eight ranked secondary endpoints in pure menstrual migraine and menstrually-related migraine. No approved treatment exists for this indication. Already-approved molecule entering a large under-treated women's-health indication, which compresses development risk and launch cost. AbbVie plans worldwide submissions; NO PDUFA date exists yet, so this is a readout row and must not be promoted to a decision row</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2301,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2288,27 +2311,27 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Ultragenyx/Abeona</t>
+          <t>Telix</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>RARE</t>
-        </is>
-      </c>
-      <c r="F32" s="2" t="inlineStr">
-        <is>
-          <t>UX111</t>
-        </is>
-      </c>
-      <c r="G32" s="2" t="inlineStr">
-        <is>
-          <t>AAV gene therapy</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
-        <is>
-          <t>Sanfilippo syndrome type A</t>
+          <t>TLX</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>TLX101-Px</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>PET imaging agent</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>glioma imaging</t>
         </is>
       </c>
       <c r="I32" s="6" t="inlineStr">
@@ -2316,56 +2339,56 @@
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K32" s="5" t="inlineStr">
-        <is>
-          <t>Second RARE gene-therapy decision in ~1 month</t>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>PDUFA date of Sep 11 2026 passed with no approval or CRL announced as of that evening; row deliberately left upcoming rather than inferred. Telix previously received a CRL on the related glioma imaging NDA TLX101-CDx, so silence is not directional</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Merck</t>
+          <t>Cullinan Therapeutics/Taiho</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
-        </is>
-      </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Winrevair (sotatercept) sNDA</t>
-        </is>
-      </c>
-      <c r="G33" s="2" t="inlineStr">
-        <is>
-          <t>activin signaling inhibitor</t>
-        </is>
-      </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>PAH earlier-line (HYPERION)</t>
+          <t>CGEM</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>zipalertinib</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>EGFR exon 20 insertion tyrosine kinase inhibitor</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>first-line EGFR exon 20 insertion mutation NSCLC</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2373,14 +2396,14 @@
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K33" s="5" t="inlineStr">
-        <is>
-          <t>Label expansion</t>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3 REZILIENT3 planned interim analysis of zipalertinib plus chemotherapy, Presidential Symposium 2 at IASLC WCLC 2026 in Seoul</t>
         </is>
       </c>
     </row>
@@ -2392,52 +2415,52 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>CHMP</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Ionis</t>
+          <t>EMA</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>IONS</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>zilganersen</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="inlineStr">
-        <is>
-          <t>antisense oligonucleotide</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>Alexander disease</t>
-        </is>
-      </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K34" s="5" t="inlineStr">
-        <is>
-          <t>Approved Sep 3 2026 as ZANVASTRO, ~3 weeks ahead of PDUFA; first-ever Alexander disease therapy; PRV awarded; Ionis' first independent neurology launch</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>CHMP monthly meeting</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I34" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Sept 14-17; new opinions resume after August written procedure</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2472,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2459,27 +2482,27 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>GRAIL</t>
+          <t>FDA</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>GRAL</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Galleri MCED test</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="inlineStr">
-        <is>
-          <t>multi-cancer early detection</t>
-        </is>
-      </c>
-      <c r="H35" s="2" t="inlineStr">
-        <is>
-          <t>cancer screening</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Pediatric Advisory Committee</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -2487,14 +2510,14 @@
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K35" s="5" t="inlineStr">
-        <is>
-          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>Virtual session</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2529,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -2516,27 +2539,27 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Incyte/Mirum</t>
+          <t>Ultragenyx/Abeona</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>INCY</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>zilurgisertib</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>ALK2 inhibitor</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
-        <is>
-          <t>anemia of myelofibrosis</t>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>UX111</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>AAV gene therapy</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Sanfilippo syndrome type A</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -2544,26 +2567,26 @@
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K36" s="5" t="inlineStr">
-        <is>
-          <t>Per pdufa.bio calendar</t>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Second RARE gene-therapy decision in ~1 month</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -2573,27 +2596,27 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Biofrontera</t>
+          <t>Merck</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>BFRI</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Ameluz + RhodoLED lamp series</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>photodynamic therapy</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>actinic keratosis</t>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Winrevair (sotatercept-csrk) sBLA</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>activin signaling inhibitor</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>PAH earlier-line (HYPERION)</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -2601,26 +2624,26 @@
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J37" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K37" s="5" t="inlineStr">
-        <is>
-          <t>Device-drug combination label expansion</t>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>HYPERION-based label expansion to newly diagnosed, first-line PAH - a larger and earlier-line population than the current label. Corrected from sNDA to sBLA: sotatercept is a biologic reviewed under BLA 761363</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -2630,42 +2653,42 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Novo Nordisk</t>
+          <t>Ionis</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>NVO</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>Mim8 (denecimig)</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>FVIII-mimetic bispecific antibody</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
-        <is>
-          <t>hemophilia A</t>
-        </is>
-      </c>
-      <c r="I38" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K38" s="5" t="inlineStr">
-        <is>
-          <t>Next-gen challenger to Hemlibra</t>
+          <t>IONS</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>zilganersen</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>antisense oligonucleotide</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Alexander disease</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J38" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Approved Sep 3 2026 as ZANVASTRO, ~3 weeks ahead of PDUFA; first-ever Alexander disease therapy; PRV awarded; Ionis' first independent neurology launch</t>
         </is>
       </c>
     </row>
@@ -2677,52 +2700,52 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>AdComm</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Protagonist/Takeda</t>
+          <t>GRAIL</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>PTGX</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>rusfertide</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>hepcidin mimetic</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>polycythemia vera</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K39" s="5" t="inlineStr">
-        <is>
-          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
+          <t>GRAL</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Galleri MCED test</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>multi-cancer early detection</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>cancer screening</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>First-ever FDA AdComm on an MCED test (PMA)</t>
         </is>
       </c>
     </row>
@@ -2734,7 +2757,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-26</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2744,27 +2767,27 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Scholar Rock</t>
+          <t>Incyte/Mirum</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>SRRK</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>apitegromab</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>anti-myostatin antibody</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>spinal muscular atrophy</t>
+          <t>INCY</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>zilurgisertib</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>ALK2 inhibitor</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>anemia of myelofibrosis</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -2772,26 +2795,26 @@
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K40" s="5" t="inlineStr">
-        <is>
-          <t>US decision after EU MAA withdrawal in Aug 2026</t>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Per pdufa.bio calendar</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2801,42 +2824,42 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Priovant/Roivant</t>
+          <t>Biofrontera</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>ROIV</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>brepocitinib</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>TYK2/JAK1 inhibitor</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>dermatomyositis</t>
-        </is>
-      </c>
-      <c r="I41" s="3" t="inlineStr">
-        <is>
-          <t>approved</t>
-        </is>
-      </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K41" s="5" t="inlineStr">
-        <is>
-          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
+          <t>BFRI</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Ameluz + RhodoLED lamp series</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>photodynamic therapy</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>actinic keratosis</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Device-drug combination label expansion</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2871,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2858,27 +2881,27 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Novo Nordisk</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Tecentriq (atezolizumab)</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>PD-L1 checkpoint inhibitor</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
-        <is>
-          <t>stage III colon cancer</t>
+          <t>NVO</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Mim8 (denecimig)</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>FVIII-mimetic bispecific antibody</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>hemophilia A</t>
         </is>
       </c>
       <c r="I42" s="6" t="inlineStr">
@@ -2886,26 +2909,26 @@
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K42" s="5" t="inlineStr">
-        <is>
-          <t>Checkpoint expansion into adjuvant colon</t>
+      <c r="J42" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>Next-gen challenger to Hemlibra</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2915,54 +2938,54 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Merck/Daiichi Sankyo</t>
+          <t>Priovant/Roivant</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>MRK</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>ifinatamab deruxtecan (DS-7300)</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>B7-H3 antibody-drug conjugate</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>extensive-stage small cell lung cancer</t>
-        </is>
-      </c>
-      <c r="I43" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K43" s="5" t="inlineStr">
-        <is>
-          <t>First regulatory decision for a B7-H3 ADC</t>
+          <t>ROIV</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>brepocitinib</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>TYK2/JAK1 inhibitor</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>dermatomyositis</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Approved Aug 27 2026 as Lisraya; first oral treatment for dermatomyositis; over a month ahead of Sep 30 PDUFA</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2972,54 +2995,54 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Roche</t>
+          <t>Protagonist/Takeda</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>RHHBY</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>Enspryng (satralizumab)</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>IL-6 receptor antagonist</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>thyroid eye disease</t>
-        </is>
-      </c>
-      <c r="I44" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K44" s="5" t="inlineStr">
-        <is>
-          <t>First IL-6R challenger to Tepezza</t>
+          <t>PTGX</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>rusfertide</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>hepcidin mimetic</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>polycythemia vera</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Approved Aug 28 2026 as MIMRYLO, ~1 month early; first-in-class hepcidin mimetic; VERIFY Ph3; ~$2B opportunity; Takeda commercializes</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3029,84 +3052,84 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Pharming</t>
+          <t>Scholar Rock</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>PHAR</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>leniolisib</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>PI3K-delta inhibitor</t>
-        </is>
-      </c>
-      <c r="H45" s="2" t="inlineStr">
-        <is>
-          <t>activated PI3K-delta syndrome (APDS)</t>
-        </is>
-      </c>
-      <c r="I45" s="6" t="inlineStr">
-        <is>
-          <t>upcoming</t>
-        </is>
-      </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K45" s="5" t="inlineStr">
-        <is>
-          <t>Label expansion for Joenja</t>
+          <t>SRRK</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>apitegromab</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr">
+        <is>
+          <t>anti-myostatin antibody</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>spinal muscular atrophy</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Approved Sep 11 2026 as ISEMBYLD (apitegromab-mstn), 19 days ahead of the Sep 30 PDUFA; first and only muscle-targeted therapy for SMA; label requires concurrent SMN2-targeted treatment, so it is add-on value on top of nusinersen/risdiplam rather than a substitution; first regulatory proof point for anti-latent-myostatin mechanism, read-through to obesity muscle-preservation programs</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>PDUFA</t>
+          <t>readout</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
+          <t>Vertex</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>GSK</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>bepirovirsen</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>antisense oligonucleotide</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
-        <is>
-          <t>chronic hepatitis B</t>
+          <t>VRTX</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>inaxaplin (VX-147)</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>APOL1 channel function inhibitor</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>APOL1-mediated kidney disease</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
@@ -3114,76 +3137,528 @@
           <t>upcoming</t>
         </is>
       </c>
-      <c r="J46" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K46" s="5" t="inlineStr">
-        <is>
-          <t>B-Well program; functional-cure ambition in HBV</t>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Phase 3 pivotal readout; would be the first precision-medicine approach in APOL1 nephropathy. Date from a third-party research calendar, not a company 8-K, so treat as a window</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>AdComm</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>FDA</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>Vaccines and Related Biological Products Advisory Committee</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
+        <is>
+          <t>influenza vaccines</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>strain selection for the 2027 Southern Hemisphere influenza season</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>Meeting 9:00 a.m. to 1:00 p.m. ET. Sourced to a dated Federal Register notice published Sep 9 2026, deliberately NOT to an aggregator calendar - the fabricated AdComm row removed on Sep 4 came from an undated archive page listing 2019-2020 meetings including a 2020 Southern Hemisphere influenza session</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>Tecentriq (atezolizumab)</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>PD-L1 checkpoint inhibitor</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>stage III colon cancer</t>
+        </is>
+      </c>
+      <c r="I48" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Checkpoint expansion into adjuvant colon</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Merck/Daiichi Sankyo</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>ifinatamab deruxtecan (DS-7300)</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>B7-H3 antibody-drug conjugate</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>extensive-stage small cell lung cancer</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>First regulatory decision for a B7-H3 ADC</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Roche</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>RHHBY</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>Enspryng (satralizumab)</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>IL-6 receptor antagonist</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>thyroid eye disease</t>
+        </is>
+      </c>
+      <c r="I50" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>First IL-6R challenger to Tepezza</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Viatris/Opus Genetics</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>VTRS</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>MR-141 (phentolamine ophthalmic solution 0.75%)</t>
+        </is>
+      </c>
+      <c r="G51" s="3" t="inlineStr">
+        <is>
+          <t>alpha-adrenergic antagonist eye drop</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>presbyopia</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>sNDA for a product already marketed as RYZUMVI. ONE row deliberately, not two: pdufa.bio lists VTRS MR-141 and IRD phentolamine 0.75% as separate Oct 17 decisions but Viatris and Opus Genetics announced the same application with the same goal date on Feb 25 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-24</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Pharming</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>PHAR</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>leniolisib</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>PI3K-delta inhibitor</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>activated PI3K-delta syndrome (APDS)</t>
+        </is>
+      </c>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Approved Sep 11 2026 for children aged 4-11 with APDS weighing at least 27 kg, 43 days ahead of the Oct 24 PDUFA; first treatment for this age group; follows an earlier CRL on this sNDA with the resubmission only accepted Jun 4 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>GSK</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>GSK</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>bepirovirsen</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>antisense oligonucleotide</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>chronic hepatitis B</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>B-Well program; functional-cure ambition in HBV</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>PDUFA</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Inovio</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>INO</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>INO-3107</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>DNA immunotherapy targeting HPV-6 and HPV-11</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>recurrent respiratory papillomatosis</t>
+        </is>
+      </c>
+      <c r="I54" s="6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>Inovio's first BLA. Indication corrected against the sponsor: TheraRadar lists this decision under cervical intraepithelial neoplasia, which would have made it a false women's-health row; INO-3107 is for RRP</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B47" s="2" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>2026-11-22</t>
         </is>
       </c>
-      <c r="C47" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>PDUFA</t>
         </is>
       </c>
-      <c r="D47" s="2" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>Capricor</t>
         </is>
       </c>
-      <c r="E47" s="2" t="inlineStr">
+      <c r="E55" s="2" t="inlineStr">
         <is>
           <t>CAPR</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr">
+      <c r="F55" s="3" t="inlineStr">
         <is>
           <t>deramiocel</t>
         </is>
       </c>
-      <c r="G47" s="2" t="inlineStr">
+      <c r="G55" s="3" t="inlineStr">
         <is>
           <t>allogeneic cell therapy</t>
         </is>
       </c>
-      <c r="H47" s="2" t="inlineStr">
+      <c r="H55" s="3" t="inlineStr">
         <is>
           <t>DMD cardiomyopathy</t>
         </is>
       </c>
-      <c r="I47" s="8" t="inlineStr">
+      <c r="I55" s="9" t="inlineStr">
         <is>
           <t>delayed</t>
         </is>
       </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="K47" s="5" t="inlineStr">
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
         <is>
           <t>PDUFA extended from Aug 22 to Nov 22 2026 after FDA accepted 24-month HOPE-3 data as major amendment; AdComm voted 9-3 against in July</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K47"/>
+  <autoFilter ref="A1:K55"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J3" r:id="rId2"/>
@@ -3231,6 +3706,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId54"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>